<commit_message>
Job refresh 2026-10-19 12:29 UTC
</commit_message>
<xml_diff>
--- a/Werkstudent_Job_Tracker.xlsx
+++ b/Werkstudent_Job_Tracker.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Excluded" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Jobs'!$A$1:$O$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Jobs'!$A$1:$O$14</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1" iterateDelta="0.0001"/>
 </workbook>
@@ -128,7 +128,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -178,6 +178,18 @@
     </xf>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -585,10 +597,10 @@
       </c>
     </row>
     <row r="2" ht="15" customHeight="1">
-      <c r="A2" s="13" t="n">
+      <c r="A2" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="13">
+      <c r="B2" s="20">
         <f>IF(OR(ISNUMBER(SEARCH("düsseldorf",E2)),ISNUMBER(SEARCH("duesseldorf",E2)),ISNUMBER(SEARCH("dusseldorf",E2)),ISNUMBER(SEARCH("köln",E2)),ISNUMBER(SEARCH("koeln",E2)),ISNUMBER(SEARCH("koln",E2)),ISNUMBER(SEARCH("cologne",E2)),ISNUMBER(SEARCH("hannover",E2)),ISNUMBER(SEARCH("hanover",E2)),ISNUMBER(SEARCH("hamburg",E2)),ISNUMBER(SEARCH("aachen",E2)),ISNUMBER(SEARCH("münchen",E2)),ISNUMBER(SEARCH("muenchen",E2)),ISNUMBER(SEARCH("munich",E2)),ISNUMBER(SEARCH("frankfurt",E2))),"1 Target city",IF(OR(E2="",E2="Verify"),"2 Verify location","3 Other city"))</f>
         <v/>
       </c>
@@ -599,43 +611,43 @@
       </c>
       <c r="D2" s="14" t="inlineStr">
         <is>
-          <t>Werkstudent/in Data Analytics &amp; Growth Insights (m/w/d) - Stepstone</t>
+          <t>Werkstudent:in Business Intelligence, Analytics und AI (m/w/d)* | XING Jobs</t>
         </is>
       </c>
       <c r="E2" s="14" t="inlineStr">
         <is>
-          <t>Köln</t>
-        </is>
-      </c>
-      <c r="F2" s="13" t="inlineStr">
+          <t>Hamburg / Köln</t>
+        </is>
+      </c>
+      <c r="F2" s="20" t="inlineStr">
         <is>
           <t>Not stated</t>
         </is>
       </c>
-      <c r="G2" s="13" t="inlineStr">
-        <is>
-          <t>StepStone</t>
-        </is>
-      </c>
-      <c r="H2" s="15" t="n">
-        <v>46311</v>
-      </c>
-      <c r="I2" s="16">
+      <c r="G2" s="20" t="inlineStr">
+        <is>
+          <t>XING</t>
+        </is>
+      </c>
+      <c r="H2" s="21" t="n">
+        <v>46314</v>
+      </c>
+      <c r="I2" s="22">
         <f>IF(H2="","",TODAY()-H2)</f>
         <v/>
       </c>
-      <c r="J2" s="13" t="inlineStr">
+      <c r="J2" s="20" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="K2" s="13" t="inlineStr">
+      <c r="K2" s="20" t="inlineStr">
         <is>
           <t>Not applied</t>
         </is>
       </c>
-      <c r="L2" s="15" t="n"/>
-      <c r="M2" s="17" t="inlineStr">
+      <c r="L2" s="21" t="n"/>
+      <c r="M2" s="23" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -645,15 +657,15 @@
           <t>Auto-added; verify company, location and requirements</t>
         </is>
       </c>
-      <c r="O2" s="15" t="n">
-        <v>46313</v>
+      <c r="O2" s="21" t="n">
+        <v>46314</v>
       </c>
     </row>
     <row r="3" ht="23.85" customHeight="1">
-      <c r="A3" s="13" t="n">
+      <c r="A3" s="20" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="13">
+      <c r="B3" s="20">
         <f>IF(OR(ISNUMBER(SEARCH("düsseldorf",E3)),ISNUMBER(SEARCH("duesseldorf",E3)),ISNUMBER(SEARCH("dusseldorf",E3)),ISNUMBER(SEARCH("köln",E3)),ISNUMBER(SEARCH("koeln",E3)),ISNUMBER(SEARCH("koln",E3)),ISNUMBER(SEARCH("cologne",E3)),ISNUMBER(SEARCH("hannover",E3)),ISNUMBER(SEARCH("hanover",E3)),ISNUMBER(SEARCH("hamburg",E3)),ISNUMBER(SEARCH("aachen",E3)),ISNUMBER(SEARCH("münchen",E3)),ISNUMBER(SEARCH("muenchen",E3)),ISNUMBER(SEARCH("munich",E3)),ISNUMBER(SEARCH("frankfurt",E3))),"1 Target city",IF(OR(E3="",E3="Verify"),"2 Verify location","3 Other city"))</f>
         <v/>
       </c>
@@ -664,61 +676,61 @@
       </c>
       <c r="D3" s="14" t="inlineStr">
         <is>
-          <t>Werkstudent:in Power BI &amp; Controlling Analytics - HDI Group</t>
+          <t>Data Analytics Intern - 6 Months - Ausbildung, Studium, Teilzeit Job in ...</t>
         </is>
       </c>
       <c r="E3" s="14" t="inlineStr">
         <is>
-          <t>Düsseldorf</t>
-        </is>
-      </c>
-      <c r="F3" s="13" t="inlineStr">
+          <t>Düsseldorf / Frankfurt am Main / Hamburg / München</t>
+        </is>
+      </c>
+      <c r="F3" s="20" t="inlineStr">
         <is>
           <t>Not stated</t>
         </is>
       </c>
-      <c r="G3" s="13" t="inlineStr">
-        <is>
-          <t>LinkedIn</t>
-        </is>
-      </c>
-      <c r="H3" s="15" t="n">
-        <v>46309</v>
-      </c>
-      <c r="I3" s="16">
+      <c r="G3" s="20" t="inlineStr">
+        <is>
+          <t>StepStone</t>
+        </is>
+      </c>
+      <c r="H3" s="21" t="n">
+        <v>46312</v>
+      </c>
+      <c r="I3" s="22">
         <f>IF(H3="","",TODAY()-H3)</f>
         <v/>
       </c>
-      <c r="J3" s="13" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="K3" s="13" t="inlineStr">
+      <c r="J3" s="20" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="K3" s="20" t="inlineStr">
         <is>
           <t>Not applied</t>
         </is>
       </c>
-      <c r="L3" s="15" t="n"/>
-      <c r="M3" s="17" t="inlineStr">
+      <c r="L3" s="21" t="n"/>
+      <c r="M3" s="23" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
       <c r="N3" s="14" t="inlineStr">
         <is>
-          <t>Auto-added; verify company, location and requirements; page content unavailable; matched search snippet only</t>
-        </is>
-      </c>
-      <c r="O3" s="15" t="n">
-        <v>46313</v>
+          <t>Auto-added; verify company, location and requirements</t>
+        </is>
+      </c>
+      <c r="O3" s="21" t="n">
+        <v>46314</v>
       </c>
     </row>
     <row r="4" ht="23.85" customHeight="1">
-      <c r="A4" s="13" t="n">
+      <c r="A4" s="20" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="13">
+      <c r="B4" s="20">
         <f>IF(OR(ISNUMBER(SEARCH("düsseldorf",E4)),ISNUMBER(SEARCH("duesseldorf",E4)),ISNUMBER(SEARCH("dusseldorf",E4)),ISNUMBER(SEARCH("köln",E4)),ISNUMBER(SEARCH("koeln",E4)),ISNUMBER(SEARCH("koln",E4)),ISNUMBER(SEARCH("cologne",E4)),ISNUMBER(SEARCH("hannover",E4)),ISNUMBER(SEARCH("hanover",E4)),ISNUMBER(SEARCH("hamburg",E4)),ISNUMBER(SEARCH("aachen",E4)),ISNUMBER(SEARCH("münchen",E4)),ISNUMBER(SEARCH("muenchen",E4)),ISNUMBER(SEARCH("munich",E4)),ISNUMBER(SEARCH("frankfurt",E4))),"1 Target city",IF(OR(E4="",E4="Verify"),"2 Verify location","3 Other city"))</f>
         <v/>
       </c>
@@ -729,225 +741,705 @@
       </c>
       <c r="D4" s="14" t="inlineStr">
         <is>
-          <t>Werkstudent:in Power BI &amp; Controlling Analytics bei HDI Group</t>
+          <t>Werkstudent/in Data Analytics &amp; Growth Insights (m/w/d) - Stepstone</t>
         </is>
       </c>
       <c r="E4" s="14" t="inlineStr">
         <is>
-          <t>Düsseldorf</t>
-        </is>
-      </c>
-      <c r="F4" s="13" t="inlineStr">
+          <t>Köln</t>
+        </is>
+      </c>
+      <c r="F4" s="20" t="inlineStr">
         <is>
           <t>Not stated</t>
         </is>
       </c>
-      <c r="G4" s="13" t="inlineStr">
-        <is>
-          <t>LinkedIn</t>
-        </is>
-      </c>
-      <c r="H4" s="15" t="n">
-        <v>46309</v>
-      </c>
-      <c r="I4" s="16">
+      <c r="G4" s="20" t="inlineStr">
+        <is>
+          <t>StepStone</t>
+        </is>
+      </c>
+      <c r="H4" s="21" t="n">
+        <v>46311</v>
+      </c>
+      <c r="I4" s="22">
         <f>IF(H4="","",TODAY()-H4)</f>
         <v/>
       </c>
-      <c r="J4" s="13" t="inlineStr">
+      <c r="J4" s="20" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="K4" s="20" t="inlineStr">
+        <is>
+          <t>Not applied</t>
+        </is>
+      </c>
+      <c r="L4" s="21" t="n"/>
+      <c r="M4" s="23" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N4" s="14" t="inlineStr">
+        <is>
+          <t>Auto-added; verify company, location and requirements</t>
+        </is>
+      </c>
+      <c r="O4" s="21" t="n">
+        <v>46313</v>
+      </c>
+    </row>
+    <row r="5" ht="23.85" customHeight="1">
+      <c r="A5" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="20">
+        <f>IF(OR(ISNUMBER(SEARCH("düsseldorf",E5)),ISNUMBER(SEARCH("duesseldorf",E5)),ISNUMBER(SEARCH("dusseldorf",E5)),ISNUMBER(SEARCH("köln",E5)),ISNUMBER(SEARCH("koeln",E5)),ISNUMBER(SEARCH("koln",E5)),ISNUMBER(SEARCH("cologne",E5)),ISNUMBER(SEARCH("hannover",E5)),ISNUMBER(SEARCH("hanover",E5)),ISNUMBER(SEARCH("hamburg",E5)),ISNUMBER(SEARCH("aachen",E5)),ISNUMBER(SEARCH("münchen",E5)),ISNUMBER(SEARCH("muenchen",E5)),ISNUMBER(SEARCH("munich",E5)),ISNUMBER(SEARCH("frankfurt",E5))),"1 Target city",IF(OR(E5="",E5="Verify"),"2 Verify location","3 Other city"))</f>
+        <v/>
+      </c>
+      <c r="C5" s="14" t="inlineStr">
+        <is>
+          <t>See link</t>
+        </is>
+      </c>
+      <c r="D5" s="14" t="inlineStr">
+        <is>
+          <t>Praktikant Business Analytics Bankenkooperation (m/w/d)</t>
+        </is>
+      </c>
+      <c r="E5" s="14" t="inlineStr">
+        <is>
+          <t>Düsseldorf</t>
+        </is>
+      </c>
+      <c r="F5" s="20" t="inlineStr">
+        <is>
+          <t>Not stated</t>
+        </is>
+      </c>
+      <c r="G5" s="20" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="H5" s="21" t="n">
+        <v>46314</v>
+      </c>
+      <c r="I5" s="22">
+        <f>IF(H5="","",TODAY()-H5)</f>
+        <v/>
+      </c>
+      <c r="J5" s="20" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="K4" s="13" t="inlineStr">
+      <c r="K5" s="20" t="inlineStr">
         <is>
           <t>Not applied</t>
         </is>
       </c>
-      <c r="L4" s="15" t="n"/>
-      <c r="M4" s="17" t="inlineStr">
+      <c r="L5" s="21" t="n"/>
+      <c r="M5" s="23" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="N4" s="14" t="inlineStr">
+      <c r="N5" s="14" t="inlineStr">
         <is>
           <t>Auto-added; verify company, location and requirements; page content unavailable; matched search snippet only</t>
         </is>
       </c>
-      <c r="O4" s="15" t="n">
+      <c r="O5" s="21" t="n">
+        <v>46314</v>
+      </c>
+    </row>
+    <row r="6" ht="23.85" customHeight="1">
+      <c r="A6" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="20">
+        <f>IF(OR(ISNUMBER(SEARCH("düsseldorf",E6)),ISNUMBER(SEARCH("duesseldorf",E6)),ISNUMBER(SEARCH("dusseldorf",E6)),ISNUMBER(SEARCH("köln",E6)),ISNUMBER(SEARCH("koeln",E6)),ISNUMBER(SEARCH("koln",E6)),ISNUMBER(SEARCH("cologne",E6)),ISNUMBER(SEARCH("hannover",E6)),ISNUMBER(SEARCH("hanover",E6)),ISNUMBER(SEARCH("hamburg",E6)),ISNUMBER(SEARCH("aachen",E6)),ISNUMBER(SEARCH("münchen",E6)),ISNUMBER(SEARCH("muenchen",E6)),ISNUMBER(SEARCH("munich",E6)),ISNUMBER(SEARCH("frankfurt",E6))),"1 Target city",IF(OR(E6="",E6="Verify"),"2 Verify location","3 Other city"))</f>
+        <v/>
+      </c>
+      <c r="C6" s="14" t="inlineStr">
+        <is>
+          <t>See link</t>
+        </is>
+      </c>
+      <c r="D6" s="14" t="inlineStr">
+        <is>
+          <t>Werkstudent:in Business &amp; Data Analyst Consultant (m/w/d)</t>
+        </is>
+      </c>
+      <c r="E6" s="14" t="inlineStr">
+        <is>
+          <t>Düsseldorf / Köln</t>
+        </is>
+      </c>
+      <c r="F6" s="20" t="inlineStr">
+        <is>
+          <t>Not stated</t>
+        </is>
+      </c>
+      <c r="G6" s="20" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="H6" s="21" t="n">
+        <v>46314</v>
+      </c>
+      <c r="I6" s="22">
+        <f>IF(H6="","",TODAY()-H6)</f>
+        <v/>
+      </c>
+      <c r="J6" s="20" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="K6" s="20" t="inlineStr">
+        <is>
+          <t>Not applied</t>
+        </is>
+      </c>
+      <c r="L6" s="21" t="n"/>
+      <c r="M6" s="23" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N6" s="14" t="inlineStr">
+        <is>
+          <t>Auto-added; verify company, location and requirements; page content unavailable; matched search snippet only</t>
+        </is>
+      </c>
+      <c r="O6" s="21" t="n">
+        <v>46314</v>
+      </c>
+    </row>
+    <row r="7" ht="15" customHeight="1">
+      <c r="A7" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="20">
+        <f>IF(OR(ISNUMBER(SEARCH("düsseldorf",E7)),ISNUMBER(SEARCH("duesseldorf",E7)),ISNUMBER(SEARCH("dusseldorf",E7)),ISNUMBER(SEARCH("köln",E7)),ISNUMBER(SEARCH("koeln",E7)),ISNUMBER(SEARCH("koln",E7)),ISNUMBER(SEARCH("cologne",E7)),ISNUMBER(SEARCH("hannover",E7)),ISNUMBER(SEARCH("hanover",E7)),ISNUMBER(SEARCH("hamburg",E7)),ISNUMBER(SEARCH("aachen",E7)),ISNUMBER(SEARCH("münchen",E7)),ISNUMBER(SEARCH("muenchen",E7)),ISNUMBER(SEARCH("munich",E7)),ISNUMBER(SEARCH("frankfurt",E7))),"1 Target city",IF(OR(E7="",E7="Verify"),"2 Verify location","3 Other city"))</f>
+        <v/>
+      </c>
+      <c r="C7" s="14" t="inlineStr">
+        <is>
+          <t>See link</t>
+        </is>
+      </c>
+      <c r="D7" s="14" t="inlineStr">
+        <is>
+          <t>Praktikum Data Science / Data Analytics &amp; BI (w/m/d)</t>
+        </is>
+      </c>
+      <c r="E7" s="14" t="inlineStr">
+        <is>
+          <t>Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="F7" s="20" t="inlineStr">
+        <is>
+          <t>Not stated</t>
+        </is>
+      </c>
+      <c r="G7" s="20" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="H7" s="21" t="n">
+        <v>46314</v>
+      </c>
+      <c r="I7" s="22">
+        <f>IF(H7="","",TODAY()-H7)</f>
+        <v/>
+      </c>
+      <c r="J7" s="20" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="K7" s="20" t="inlineStr">
+        <is>
+          <t>Not applied</t>
+        </is>
+      </c>
+      <c r="L7" s="21" t="n"/>
+      <c r="M7" s="23" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N7" s="14" t="inlineStr">
+        <is>
+          <t>Auto-added; verify company, location and requirements; page content unavailable; matched search snippet only</t>
+        </is>
+      </c>
+      <c r="O7" s="21" t="n">
+        <v>46314</v>
+      </c>
+    </row>
+    <row r="8" ht="15" customHeight="1">
+      <c r="A8" s="20" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="20">
+        <f>IF(OR(ISNUMBER(SEARCH("düsseldorf",E8)),ISNUMBER(SEARCH("duesseldorf",E8)),ISNUMBER(SEARCH("dusseldorf",E8)),ISNUMBER(SEARCH("köln",E8)),ISNUMBER(SEARCH("koeln",E8)),ISNUMBER(SEARCH("koln",E8)),ISNUMBER(SEARCH("cologne",E8)),ISNUMBER(SEARCH("hannover",E8)),ISNUMBER(SEARCH("hanover",E8)),ISNUMBER(SEARCH("hamburg",E8)),ISNUMBER(SEARCH("aachen",E8)),ISNUMBER(SEARCH("münchen",E8)),ISNUMBER(SEARCH("muenchen",E8)),ISNUMBER(SEARCH("munich",E8)),ISNUMBER(SEARCH("frankfurt",E8))),"1 Target city",IF(OR(E8="",E8="Verify"),"2 Verify location","3 Other city"))</f>
+        <v/>
+      </c>
+      <c r="C8" s="14" t="inlineStr">
+        <is>
+          <t>See link</t>
+        </is>
+      </c>
+      <c r="D8" s="14" t="inlineStr">
+        <is>
+          <t>Praktikant Marktforschung - Business Intelligence &amp; Analytics (w/m/d)</t>
+        </is>
+      </c>
+      <c r="E8" s="14" t="inlineStr">
+        <is>
+          <t>Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="F8" s="20" t="inlineStr">
+        <is>
+          <t>Not stated</t>
+        </is>
+      </c>
+      <c r="G8" s="20" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="H8" s="21" t="n">
         <v>46313</v>
       </c>
-    </row>
-    <row r="5" ht="23.85" customHeight="1">
-      <c r="A5" s="8" t="n"/>
-      <c r="B5" s="8" t="n"/>
-      <c r="C5" s="9" t="n"/>
-      <c r="D5" s="9" t="n"/>
-      <c r="E5" s="9" t="n"/>
-      <c r="F5" s="8" t="n"/>
-      <c r="G5" s="8" t="n"/>
-      <c r="H5" s="18" t="n"/>
-      <c r="I5" s="11" t="n"/>
-      <c r="J5" s="8" t="n"/>
-      <c r="K5" s="8" t="n"/>
-      <c r="L5" s="18" t="n"/>
-      <c r="M5" s="12" t="n"/>
-      <c r="N5" s="9" t="n"/>
-      <c r="O5" s="18" t="n"/>
-    </row>
-    <row r="6" ht="23.85" customHeight="1">
-      <c r="A6" s="8" t="n"/>
-      <c r="B6" s="8" t="n"/>
-      <c r="C6" s="9" t="n"/>
-      <c r="D6" s="9" t="n"/>
-      <c r="E6" s="9" t="n"/>
-      <c r="F6" s="8" t="n"/>
-      <c r="G6" s="8" t="n"/>
-      <c r="H6" s="18" t="n"/>
-      <c r="I6" s="11" t="n"/>
-      <c r="J6" s="8" t="n"/>
-      <c r="K6" s="8" t="n"/>
-      <c r="L6" s="18" t="n"/>
-      <c r="M6" s="12" t="n"/>
-      <c r="N6" s="9" t="n"/>
-      <c r="O6" s="18" t="n"/>
-    </row>
-    <row r="7" ht="15" customHeight="1">
-      <c r="A7" s="8" t="n"/>
-      <c r="B7" s="8" t="n"/>
-      <c r="C7" s="9" t="n"/>
-      <c r="D7" s="9" t="n"/>
-      <c r="E7" s="9" t="n"/>
-      <c r="F7" s="8" t="n"/>
-      <c r="G7" s="8" t="n"/>
-      <c r="H7" s="18" t="n"/>
-      <c r="I7" s="11" t="n"/>
-      <c r="J7" s="8" t="n"/>
-      <c r="K7" s="8" t="n"/>
-      <c r="L7" s="18" t="n"/>
-      <c r="M7" s="12" t="n"/>
-      <c r="N7" s="9" t="n"/>
-      <c r="O7" s="18" t="n"/>
-    </row>
-    <row r="8" ht="15" customHeight="1">
-      <c r="A8" s="8" t="n"/>
-      <c r="B8" s="8" t="n"/>
-      <c r="C8" s="9" t="n"/>
-      <c r="D8" s="9" t="n"/>
-      <c r="E8" s="9" t="n"/>
-      <c r="F8" s="8" t="n"/>
-      <c r="G8" s="8" t="n"/>
-      <c r="H8" s="18" t="n"/>
-      <c r="I8" s="11" t="n"/>
-      <c r="J8" s="8" t="n"/>
-      <c r="K8" s="8" t="n"/>
-      <c r="L8" s="18" t="n"/>
-      <c r="M8" s="12" t="n"/>
-      <c r="N8" s="9" t="n"/>
-      <c r="O8" s="18" t="n"/>
+      <c r="I8" s="22">
+        <f>IF(H8="","",TODAY()-H8)</f>
+        <v/>
+      </c>
+      <c r="J8" s="20" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="K8" s="20" t="inlineStr">
+        <is>
+          <t>Not applied</t>
+        </is>
+      </c>
+      <c r="L8" s="21" t="n"/>
+      <c r="M8" s="23" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N8" s="14" t="inlineStr">
+        <is>
+          <t>Auto-added; verify company, location and requirements; page content unavailable; matched search snippet only</t>
+        </is>
+      </c>
+      <c r="O8" s="21" t="n">
+        <v>46314</v>
+      </c>
     </row>
     <row r="9" ht="15" customHeight="1">
-      <c r="A9" s="8" t="n"/>
-      <c r="B9" s="8" t="n"/>
-      <c r="C9" s="9" t="n"/>
-      <c r="D9" s="9" t="n"/>
-      <c r="E9" s="9" t="n"/>
-      <c r="F9" s="8" t="n"/>
-      <c r="G9" s="8" t="n"/>
-      <c r="H9" s="18" t="n"/>
-      <c r="I9" s="11" t="n"/>
-      <c r="J9" s="8" t="n"/>
-      <c r="K9" s="8" t="n"/>
-      <c r="L9" s="18" t="n"/>
-      <c r="M9" s="12" t="n"/>
-      <c r="N9" s="9" t="n"/>
-      <c r="O9" s="18" t="n"/>
+      <c r="A9" s="20" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="20">
+        <f>IF(OR(ISNUMBER(SEARCH("düsseldorf",E9)),ISNUMBER(SEARCH("duesseldorf",E9)),ISNUMBER(SEARCH("dusseldorf",E9)),ISNUMBER(SEARCH("köln",E9)),ISNUMBER(SEARCH("koeln",E9)),ISNUMBER(SEARCH("koln",E9)),ISNUMBER(SEARCH("cologne",E9)),ISNUMBER(SEARCH("hannover",E9)),ISNUMBER(SEARCH("hanover",E9)),ISNUMBER(SEARCH("hamburg",E9)),ISNUMBER(SEARCH("aachen",E9)),ISNUMBER(SEARCH("münchen",E9)),ISNUMBER(SEARCH("muenchen",E9)),ISNUMBER(SEARCH("munich",E9)),ISNUMBER(SEARCH("frankfurt",E9))),"1 Target city",IF(OR(E9="",E9="Verify"),"2 Verify location","3 Other city"))</f>
+        <v/>
+      </c>
+      <c r="C9" s="14" t="inlineStr">
+        <is>
+          <t>See link</t>
+        </is>
+      </c>
+      <c r="D9" s="14" t="inlineStr">
+        <is>
+          <t>Werkstudent:in KI &amp; Data Engineering (m/w/d)</t>
+        </is>
+      </c>
+      <c r="E9" s="14" t="inlineStr">
+        <is>
+          <t>Köln</t>
+        </is>
+      </c>
+      <c r="F9" s="20" t="inlineStr">
+        <is>
+          <t>Not stated</t>
+        </is>
+      </c>
+      <c r="G9" s="20" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="H9" s="21" t="n">
+        <v>46312</v>
+      </c>
+      <c r="I9" s="22">
+        <f>IF(H9="","",TODAY()-H9)</f>
+        <v/>
+      </c>
+      <c r="J9" s="20" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="K9" s="20" t="inlineStr">
+        <is>
+          <t>Not applied</t>
+        </is>
+      </c>
+      <c r="L9" s="21" t="n"/>
+      <c r="M9" s="23" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N9" s="14" t="inlineStr">
+        <is>
+          <t>Auto-added; verify company, location and requirements; page content unavailable; matched search snippet only</t>
+        </is>
+      </c>
+      <c r="O9" s="21" t="n">
+        <v>46314</v>
+      </c>
     </row>
     <row r="10" ht="15" customHeight="1">
-      <c r="A10" s="8" t="n"/>
-      <c r="B10" s="8" t="n"/>
-      <c r="C10" s="9" t="n"/>
-      <c r="D10" s="9" t="n"/>
-      <c r="E10" s="9" t="n"/>
-      <c r="F10" s="8" t="n"/>
-      <c r="G10" s="8" t="n"/>
-      <c r="H10" s="18" t="n"/>
-      <c r="I10" s="11" t="n"/>
-      <c r="J10" s="8" t="n"/>
-      <c r="K10" s="8" t="n"/>
-      <c r="L10" s="18" t="n"/>
-      <c r="M10" s="12" t="n"/>
-      <c r="N10" s="9" t="n"/>
-      <c r="O10" s="18" t="n"/>
+      <c r="A10" s="20" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="20">
+        <f>IF(OR(ISNUMBER(SEARCH("düsseldorf",E10)),ISNUMBER(SEARCH("duesseldorf",E10)),ISNUMBER(SEARCH("dusseldorf",E10)),ISNUMBER(SEARCH("köln",E10)),ISNUMBER(SEARCH("koeln",E10)),ISNUMBER(SEARCH("koln",E10)),ISNUMBER(SEARCH("cologne",E10)),ISNUMBER(SEARCH("hannover",E10)),ISNUMBER(SEARCH("hanover",E10)),ISNUMBER(SEARCH("hamburg",E10)),ISNUMBER(SEARCH("aachen",E10)),ISNUMBER(SEARCH("münchen",E10)),ISNUMBER(SEARCH("muenchen",E10)),ISNUMBER(SEARCH("munich",E10)),ISNUMBER(SEARCH("frankfurt",E10))),"1 Target city",IF(OR(E10="",E10="Verify"),"2 Verify location","3 Other city"))</f>
+        <v/>
+      </c>
+      <c r="C10" s="14" t="inlineStr">
+        <is>
+          <t>See link</t>
+        </is>
+      </c>
+      <c r="D10" s="14" t="inlineStr">
+        <is>
+          <t>Werkstudent Business Intelligence &amp; Analytics (m/w/d)</t>
+        </is>
+      </c>
+      <c r="E10" s="14" t="inlineStr">
+        <is>
+          <t>Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="F10" s="20" t="inlineStr">
+        <is>
+          <t>Not stated</t>
+        </is>
+      </c>
+      <c r="G10" s="20" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="H10" s="21" t="n">
+        <v>46312</v>
+      </c>
+      <c r="I10" s="22">
+        <f>IF(H10="","",TODAY()-H10)</f>
+        <v/>
+      </c>
+      <c r="J10" s="20" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="K10" s="20" t="inlineStr">
+        <is>
+          <t>Not applied</t>
+        </is>
+      </c>
+      <c r="L10" s="21" t="n"/>
+      <c r="M10" s="23" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N10" s="14" t="inlineStr">
+        <is>
+          <t>Auto-added; verify company, location and requirements; page content unavailable; matched search snippet only</t>
+        </is>
+      </c>
+      <c r="O10" s="21" t="n">
+        <v>46314</v>
+      </c>
     </row>
     <row r="11" ht="15" customHeight="1">
-      <c r="A11" s="8" t="n"/>
-      <c r="B11" s="8" t="n"/>
-      <c r="C11" s="9" t="n"/>
-      <c r="D11" s="9" t="n"/>
-      <c r="E11" s="9" t="n"/>
-      <c r="F11" s="8" t="n"/>
-      <c r="G11" s="8" t="n"/>
-      <c r="H11" s="18" t="n"/>
-      <c r="I11" s="11" t="n"/>
-      <c r="J11" s="8" t="n"/>
-      <c r="K11" s="8" t="n"/>
-      <c r="L11" s="18" t="n"/>
-      <c r="M11" s="12" t="n"/>
-      <c r="N11" s="9" t="n"/>
-      <c r="O11" s="18" t="n"/>
+      <c r="A11" s="20" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="20">
+        <f>IF(OR(ISNUMBER(SEARCH("düsseldorf",E11)),ISNUMBER(SEARCH("duesseldorf",E11)),ISNUMBER(SEARCH("dusseldorf",E11)),ISNUMBER(SEARCH("köln",E11)),ISNUMBER(SEARCH("koeln",E11)),ISNUMBER(SEARCH("koln",E11)),ISNUMBER(SEARCH("cologne",E11)),ISNUMBER(SEARCH("hannover",E11)),ISNUMBER(SEARCH("hanover",E11)),ISNUMBER(SEARCH("hamburg",E11)),ISNUMBER(SEARCH("aachen",E11)),ISNUMBER(SEARCH("münchen",E11)),ISNUMBER(SEARCH("muenchen",E11)),ISNUMBER(SEARCH("munich",E11)),ISNUMBER(SEARCH("frankfurt",E11))),"1 Target city",IF(OR(E11="",E11="Verify"),"2 Verify location","3 Other city"))</f>
+        <v/>
+      </c>
+      <c r="C11" s="14" t="inlineStr">
+        <is>
+          <t>See link</t>
+        </is>
+      </c>
+      <c r="D11" s="14" t="inlineStr">
+        <is>
+          <t>Werkstudent*in Data Analytics bei Union Investment</t>
+        </is>
+      </c>
+      <c r="E11" s="14" t="inlineStr">
+        <is>
+          <t>Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="F11" s="20" t="inlineStr">
+        <is>
+          <t>Not stated</t>
+        </is>
+      </c>
+      <c r="G11" s="20" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="H11" s="21" t="n">
+        <v>46312</v>
+      </c>
+      <c r="I11" s="22">
+        <f>IF(H11="","",TODAY()-H11)</f>
+        <v/>
+      </c>
+      <c r="J11" s="20" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="K11" s="20" t="inlineStr">
+        <is>
+          <t>Not applied</t>
+        </is>
+      </c>
+      <c r="L11" s="21" t="n"/>
+      <c r="M11" s="23" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N11" s="14" t="inlineStr">
+        <is>
+          <t>Auto-added; verify company, location and requirements; page content unavailable; matched search snippet only</t>
+        </is>
+      </c>
+      <c r="O11" s="21" t="n">
+        <v>46314</v>
+      </c>
     </row>
     <row r="12" ht="23.85" customHeight="1">
-      <c r="A12" s="8" t="n"/>
-      <c r="B12" s="8" t="n"/>
-      <c r="C12" s="9" t="n"/>
-      <c r="D12" s="9" t="n"/>
-      <c r="E12" s="9" t="n"/>
-      <c r="F12" s="8" t="n"/>
-      <c r="G12" s="8" t="n"/>
-      <c r="H12" s="18" t="n"/>
-      <c r="I12" s="11" t="n"/>
-      <c r="J12" s="8" t="n"/>
-      <c r="K12" s="8" t="n"/>
-      <c r="L12" s="18" t="n"/>
-      <c r="M12" s="12" t="n"/>
-      <c r="N12" s="9" t="n"/>
-      <c r="O12" s="18" t="n"/>
+      <c r="A12" s="20" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="20">
+        <f>IF(OR(ISNUMBER(SEARCH("düsseldorf",E12)),ISNUMBER(SEARCH("duesseldorf",E12)),ISNUMBER(SEARCH("dusseldorf",E12)),ISNUMBER(SEARCH("köln",E12)),ISNUMBER(SEARCH("koeln",E12)),ISNUMBER(SEARCH("koln",E12)),ISNUMBER(SEARCH("cologne",E12)),ISNUMBER(SEARCH("hannover",E12)),ISNUMBER(SEARCH("hanover",E12)),ISNUMBER(SEARCH("hamburg",E12)),ISNUMBER(SEARCH("aachen",E12)),ISNUMBER(SEARCH("münchen",E12)),ISNUMBER(SEARCH("muenchen",E12)),ISNUMBER(SEARCH("munich",E12)),ISNUMBER(SEARCH("frankfurt",E12))),"1 Target city",IF(OR(E12="",E12="Verify"),"2 Verify location","3 Other city"))</f>
+        <v/>
+      </c>
+      <c r="C12" s="14" t="inlineStr">
+        <is>
+          <t>See link</t>
+        </is>
+      </c>
+      <c r="D12" s="14" t="inlineStr">
+        <is>
+          <t>Werkstudent:in Power BI &amp; Controlling Analytics - HDI Group</t>
+        </is>
+      </c>
+      <c r="E12" s="14" t="inlineStr">
+        <is>
+          <t>Düsseldorf</t>
+        </is>
+      </c>
+      <c r="F12" s="20" t="inlineStr">
+        <is>
+          <t>Not stated</t>
+        </is>
+      </c>
+      <c r="G12" s="20" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="H12" s="21" t="n">
+        <v>46309</v>
+      </c>
+      <c r="I12" s="22">
+        <f>IF(H12="","",TODAY()-H12)</f>
+        <v/>
+      </c>
+      <c r="J12" s="20" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="K12" s="20" t="inlineStr">
+        <is>
+          <t>Not applied</t>
+        </is>
+      </c>
+      <c r="L12" s="21" t="n"/>
+      <c r="M12" s="23" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N12" s="14" t="inlineStr">
+        <is>
+          <t>Auto-added; verify company, location and requirements; page content unavailable; matched search snippet only</t>
+        </is>
+      </c>
+      <c r="O12" s="21" t="n">
+        <v>46313</v>
+      </c>
     </row>
     <row r="13" ht="15" customHeight="1">
-      <c r="A13" s="8" t="n"/>
-      <c r="B13" s="8" t="n"/>
-      <c r="C13" s="9" t="n"/>
-      <c r="D13" s="9" t="n"/>
-      <c r="E13" s="9" t="n"/>
-      <c r="F13" s="8" t="n"/>
-      <c r="G13" s="8" t="n"/>
-      <c r="H13" s="18" t="n"/>
-      <c r="I13" s="11" t="n"/>
-      <c r="J13" s="8" t="n"/>
-      <c r="K13" s="8" t="n"/>
-      <c r="L13" s="18" t="n"/>
-      <c r="M13" s="12" t="n"/>
-      <c r="N13" s="9" t="n"/>
-      <c r="O13" s="18" t="n"/>
+      <c r="A13" s="20" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="20">
+        <f>IF(OR(ISNUMBER(SEARCH("düsseldorf",E13)),ISNUMBER(SEARCH("duesseldorf",E13)),ISNUMBER(SEARCH("dusseldorf",E13)),ISNUMBER(SEARCH("köln",E13)),ISNUMBER(SEARCH("koeln",E13)),ISNUMBER(SEARCH("koln",E13)),ISNUMBER(SEARCH("cologne",E13)),ISNUMBER(SEARCH("hannover",E13)),ISNUMBER(SEARCH("hanover",E13)),ISNUMBER(SEARCH("hamburg",E13)),ISNUMBER(SEARCH("aachen",E13)),ISNUMBER(SEARCH("münchen",E13)),ISNUMBER(SEARCH("muenchen",E13)),ISNUMBER(SEARCH("munich",E13)),ISNUMBER(SEARCH("frankfurt",E13))),"1 Target city",IF(OR(E13="",E13="Verify"),"2 Verify location","3 Other city"))</f>
+        <v/>
+      </c>
+      <c r="C13" s="14" t="inlineStr">
+        <is>
+          <t>See link</t>
+        </is>
+      </c>
+      <c r="D13" s="14" t="inlineStr">
+        <is>
+          <t>Werkstudent:in Power BI &amp; Controlling Analytics bei HDI Group</t>
+        </is>
+      </c>
+      <c r="E13" s="14" t="inlineStr">
+        <is>
+          <t>Düsseldorf</t>
+        </is>
+      </c>
+      <c r="F13" s="20" t="inlineStr">
+        <is>
+          <t>Not stated</t>
+        </is>
+      </c>
+      <c r="G13" s="20" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="H13" s="21" t="n">
+        <v>46309</v>
+      </c>
+      <c r="I13" s="22">
+        <f>IF(H13="","",TODAY()-H13)</f>
+        <v/>
+      </c>
+      <c r="J13" s="20" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="K13" s="20" t="inlineStr">
+        <is>
+          <t>Not applied</t>
+        </is>
+      </c>
+      <c r="L13" s="21" t="n"/>
+      <c r="M13" s="23" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N13" s="14" t="inlineStr">
+        <is>
+          <t>Auto-added; verify company, location and requirements; page content unavailable; matched search snippet only</t>
+        </is>
+      </c>
+      <c r="O13" s="21" t="n">
+        <v>46313</v>
+      </c>
     </row>
     <row r="14" ht="15" customHeight="1">
-      <c r="A14" s="8" t="n"/>
-      <c r="B14" s="8" t="n"/>
-      <c r="C14" s="9" t="n"/>
-      <c r="D14" s="9" t="n"/>
-      <c r="E14" s="9" t="n"/>
-      <c r="F14" s="8" t="n"/>
-      <c r="G14" s="8" t="n"/>
-      <c r="H14" s="18" t="n"/>
-      <c r="I14" s="11" t="n"/>
-      <c r="J14" s="8" t="n"/>
-      <c r="K14" s="8" t="n"/>
-      <c r="L14" s="18" t="n"/>
-      <c r="M14" s="12" t="n"/>
-      <c r="N14" s="9" t="n"/>
-      <c r="O14" s="18" t="n"/>
+      <c r="A14" s="20" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="20">
+        <f>IF(OR(ISNUMBER(SEARCH("düsseldorf",E14)),ISNUMBER(SEARCH("duesseldorf",E14)),ISNUMBER(SEARCH("dusseldorf",E14)),ISNUMBER(SEARCH("köln",E14)),ISNUMBER(SEARCH("koeln",E14)),ISNUMBER(SEARCH("koln",E14)),ISNUMBER(SEARCH("cologne",E14)),ISNUMBER(SEARCH("hannover",E14)),ISNUMBER(SEARCH("hanover",E14)),ISNUMBER(SEARCH("hamburg",E14)),ISNUMBER(SEARCH("aachen",E14)),ISNUMBER(SEARCH("münchen",E14)),ISNUMBER(SEARCH("muenchen",E14)),ISNUMBER(SEARCH("munich",E14)),ISNUMBER(SEARCH("frankfurt",E14))),"1 Target city",IF(OR(E14="",E14="Verify"),"2 Verify location","3 Other city"))</f>
+        <v/>
+      </c>
+      <c r="C14" s="14" t="inlineStr">
+        <is>
+          <t>See link</t>
+        </is>
+      </c>
+      <c r="D14" s="14" t="inlineStr">
+        <is>
+          <t>Werkstudent:in Business &amp; Data Analyst Consultant (m/w/d) - XING</t>
+        </is>
+      </c>
+      <c r="E14" s="14" t="inlineStr">
+        <is>
+          <t>Köln</t>
+        </is>
+      </c>
+      <c r="F14" s="20" t="inlineStr">
+        <is>
+          <t>Not stated</t>
+        </is>
+      </c>
+      <c r="G14" s="20" t="inlineStr">
+        <is>
+          <t>XING</t>
+        </is>
+      </c>
+      <c r="H14" s="21" t="n">
+        <v>46314</v>
+      </c>
+      <c r="I14" s="22">
+        <f>IF(H14="","",TODAY()-H14)</f>
+        <v/>
+      </c>
+      <c r="J14" s="20" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="K14" s="20" t="inlineStr">
+        <is>
+          <t>Not applied</t>
+        </is>
+      </c>
+      <c r="L14" s="21" t="n"/>
+      <c r="M14" s="23" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N14" s="14" t="inlineStr">
+        <is>
+          <t>Auto-added; verify company, location and requirements; check German requirement against B1</t>
+        </is>
+      </c>
+      <c r="O14" s="21" t="n">
+        <v>46314</v>
+      </c>
     </row>
     <row r="15" ht="15" customHeight="1">
       <c r="A15" s="8" t="n"/>
@@ -4452,7 +4944,7 @@
       <c r="O220" s="18" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O4"/>
+  <autoFilter ref="A1:O14"/>
   <conditionalFormatting sqref="B2:B1000">
     <cfRule type="expression" priority="5" dxfId="2">
       <formula>LEFT($B2,1)="1"</formula>
@@ -4494,6 +4986,16 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M3" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M14" r:id="rId13"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="300" verticalDpi="300"/>
@@ -4528,7 +5030,7 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>Werkstudent: Data Analysis / Business Intelligence / Data Engineering</t>
+          <t>Werkstudent / Internship: Data Analysis / Business Intelligence / Data Engineering</t>
         </is>
       </c>
     </row>
@@ -4539,7 +5041,7 @@
         </is>
       </c>
       <c r="B3" s="19" t="n">
-        <v>46313</v>
+        <v>46314</v>
       </c>
     </row>
     <row r="4" ht="15" customHeight="1">
@@ -4550,7 +5052,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Past-week search; unknown posting dates need verification</t>
+          <t>Less than 3 days old; unknown posting dates excluded</t>
         </is>
       </c>
     </row>

</xml_diff>